<commit_message>
Reels: VO mein emotion tag kam se kam, alag VO script txt, part 2 summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVfDRs8Z25TZnX8xvhD7fv
</commit_message>
<xml_diff>
--- a/youtube stories/batch 3/Batch 3 - 10 Reels.xlsx
+++ b/youtube stories/batch 3/Batch 3 - 10 Reels.xlsx
@@ -774,7 +774,7 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Reel VO poori story EK BAAR mein banti hai (Rudra, eleven_v4, stability 0.45, speed 1.05 + purana tighten). VO mein NAHI: 'bole/boli', motive line (sirf SUSPECT card par), 'ab suniye sabke bayaan', jo photo mein dikhe (jaise 'haath laal'), galat-ishara line, saboot, 'full video/link bio' line. Saboot ke time ek jagah-set line (saboot ka naam nahi): jaise 'Drawing room mein sab kuch waisa hi tha... Shivam ne har cheez par nazar daali.' End hamesha: 3 sec chup -&gt; PAKAD_LIYA_HI + CTA_HI + SIGNATURE_HI (purani files, dobara nahi banti). Bayaan mein emotion tag ([annoyed] [nervous] [calm]...), har suspect ko koi tag - killer alag na lage. Reel 55-60 sec.</t>
+          <t>Reel VO poori story EK BAAR mein (Rudra, eleven_v4, stability 0.45, speed 1.05 + purana tighten). EMOTION TAG KAM SE KAM: sirf hook par [whispers], baaki saadi line – suspect ke bayaan par koi tag nahi (killer alag na lage). VO mein NAHI: 'bole/boli', motive line, galat-ishara line, saboot ka naam, 'full video/link bio'. End: 3 sec chup -&gt; PAKAD_LIYA_HI + CTA_HI + SIGNATURE_HI (purani files, dobara nahi banti).</t>
         </is>
       </c>
     </row>
@@ -2320,16 +2320,16 @@
         <is>
           <t>[whispers] पाँच लोग। पाँच शहर। एक झूठा सफ़र।
 रायपुर। मिल मालिक कमलेश अग्रवाल, अपने बंगले के स्टडी रूम में मरे मिले!
-[serious] मौत रात आठ से नौ के बीच। घर के सब लोग बोले, हम तो शहर से बाहर थे।
+मौत रात आठ से नौ के बीच। घर के सब लोग बोले, हम तो शहर से बाहर थे।
 डिटेक्टिव शिवम बंगले पहुँचे।
-[thoughtful] स्टडी रूम में सफ़र की तस्वीरें लगी थीं। शिवम ने हर चीज़ पर नज़र डाली।
-बेटा राहुल... [annoyed] "मैं हैदराबाद में था। हुसैन सागर झील में बुद्ध की बड़ी मूर्ति के पास बोटिंग कर रहा था।"
-मैनेजर जोशी... [nervous] "मैं आगरा में था। यमुना किनारे ताज महल देखकर लौटा।"
-भाई नरेश... [excited] "मैं दिल्ली में था। क़ुतुब मीनार देख रहा था... शाहजहाँ ने क्या कमाल की चीज़ बनवाई है!"
-ड्राइवर बबलू... [nervous] "मैं जयपुर में था। गुलाबी शहर में हवा महल के सामने चाय पी।"
-भतीजी अदिति... [calm] "मैं मैसूर में थी। मैसूर पैलेस की रोशनी देख रही थी।"
+स्टडी रूम में सफ़र की तस्वीरें लगी थीं। शिवम ने हर चीज़ पर नज़र डाली।
+बेटा राहुल... "मैं हैदराबाद में था। हुसैन सागर झील में बुद्ध की बड़ी मूर्ति के पास बोटिंग कर रहा था।"
+मैनेजर जोशी... "मैं आगरा में था। यमुना किनारे ताज महल देखकर लौटा।"
+भाई नरेश... "मैं दिल्ली में था। क़ुतुब मीनार देख रहा था... शाहजहाँ ने क्या कमाल की चीज़ बनवाई है!"
+ड्राइवर बबलू... "मैं जयपुर में था। गुलाबी शहर में हवा महल के सामने चाय पी।"
+भतीजी अदिति... "मैं मैसूर में थी। मैसूर पैलेस की रोशनी देख रही थी।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2395,16 +2395,16 @@
         <is>
           <t>[whispers] पाँच लोग। पाँच किनारे। एक ग़लत लहर।
 विशाखापट्टनम। रिज़ॉर्ट मालिक श्रीनिवास राव, अपने ऑफ़िस में मरे मिले!
-[serious] मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग समुंदर किनारे छुट्टी पर थे।
+मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग समुंदर किनारे छुट्टी पर थे।
 डिटेक्टिव शिवम रिज़ॉर्ट पहुँचे।
-[thoughtful] ऑफ़िस में समुंदर की हवा आ रही थी। शिवम ने हर चीज़ पर नज़र डाली।
-पार्टनर रेड्डी... [annoyed] "मैं गोवा के बागा बीच पर था। अरब सागर की लहरें देख रहा था।"
-मैनेजर डिसूज़ा... [excited] "मैं ओडिशा में पुरी के बीच पर था। अरब सागर का पानी इतना साफ़ था, मज़ा आ गया!"
-पत्नी लता... [calm] "मैं कन्याकुमारी में थी, जहाँ तीन समुंदर मिलते हैं।"
-लाइफ़गार्ड जॉनी... [nervous] "मैं अंडमान के हैवलॉक द्वीप पर डाइविंग सिखा रहा था।"
-रिसेप्शनिस्ट मीना... [calm] "मैं यहीं विशाखापट्टनम के आर.के. बीच पर थी, बंगाल की खाड़ी के किनारे।"
+ऑफ़िस में समुंदर की हवा आ रही थी। शिवम ने हर चीज़ पर नज़र डाली।
+पार्टनर रेड्डी... "मैं गोवा के बागा बीच पर था। अरब सागर की लहरें देख रहा था।"
+मैनेजर डिसूज़ा... "मैं ओडिशा में पुरी के बीच पर था। अरब सागर का पानी इतना साफ़ था, मज़ा आ गया!"
+पत्नी लता... "मैं कन्याकुमारी में थी, जहाँ तीन समुंदर मिलते हैं।"
+लाइफ़गार्ड जॉनी... "मैं अंडमान के हैवलॉक द्वीप पर डाइविंग सिखा रहा था।"
+रिसेप्शनिस्ट मीना... "मैं यहीं विशाखापट्टनम के आर.के. बीच पर थी, बंगाल की खाड़ी के किनारे।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2470,16 +2470,16 @@
         <is>
           <t>[whispers] दस खिलाड़ी। एक खेल। एक बेईमान।
 पुणे। स्पोर्ट्स क्लब के प्रेसिडेंट विजय देशमुख, लॉकर रूम में मरे मिले!
-[serious] मौत शाम पाँच से छह के बीच। उस वक़्त क्लब में हर कोई कोई न कोई खेल खेल रहा था।
+मौत शाम पाँच से छह के बीच। उस वक़्त क्लब में हर कोई कोई न कोई खेल खेल रहा था।
 डिटेक्टिव शिवम क्लब पहुँचे।
-[thoughtful] लॉकर रूम में ट्रॉफ़ियाँ बिखरी थीं। शिवम ने हर चीज़ पर नज़र डाली।
-हॉकी कोच गिल... [annoyed] "मैं मैदान पर हॉकी मैच करवा रहा था। दोनों टीमों में ग्यारह-ग्यारह खिलाड़ी।"
-कबड्डी खिलाड़ी बाला... [calm] "मैं कबड्डी खेल रहा था। कोर्ट पर हर टीम के सात खिलाड़ी।"
-फ़ुटबॉल रेफ़री मैथ्यू... [calm] "मैं फ़ुटबॉल मैच में रेफ़री था। नब्बे मिनट का पूरा मैच।"
-शतरंज खिलाड़ी विनायक... [nervous] "मैं शतरंज टूर्नामेंट में था। चौंसठ ख़ानों वाला बोर्ड।"
-वॉलीबॉल कप्तान अजिंक्य... [excited] "मैं वॉलीबॉल मैच खेल रहा था। हमारी टीम के ग्यारह के ग्यारह खिलाड़ी कोर्ट पर थे, पूरा ज़ोर लगा दिया!"
+लॉकर रूम में ट्रॉफ़ियाँ बिखरी थीं। शिवम ने हर चीज़ पर नज़र डाली।
+हॉकी कोच गिल... "मैं मैदान पर हॉकी मैच करवा रहा था। दोनों टीमों में ग्यारह-ग्यारह खिलाड़ी।"
+कबड्डी खिलाड़ी बाला... "मैं कबड्डी खेल रहा था। कोर्ट पर हर टीम के सात खिलाड़ी।"
+फ़ुटबॉल रेफ़री मैथ्यू... "मैं फ़ुटबॉल मैच में रेफ़री था। नब्बे मिनट का पूरा मैच।"
+शतरंज खिलाड़ी विनायक... "मैं शतरंज टूर्नामेंट में था। चौंसठ ख़ानों वाला बोर्ड।"
+वॉलीबॉल कप्तान अजिंक्य... "मैं वॉलीबॉल मैच खेल रहा था। हमारी टीम के ग्यारह के ग्यारह खिलाड़ी कोर्ट पर थे, पूरा ज़ोर लगा दिया!"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2545,16 +2545,16 @@
         <is>
           <t>[whispers] आठ बयान। आठ बातें। एक बात झूठी।
 जबलपुर। साइंस टीचर रमेश पांडे, अपने घर में मरे मिले!
-[serious] मौत रात आठ से नौ के बीच। घर के सब लोग अपने-अपने काम में लगे थे।
+मौत रात आठ से नौ के बीच। घर के सब लोग अपने-अपने काम में लगे थे।
 डिटेक्टिव शिवम घर पहुँचे।
-[thoughtful] घर में किताबें और ग्लोब रखे थे। शिवम ने हर चीज़ पर नज़र डाली।
-पत्नी उर्मिला... [calm] "मैं रसोई में दाल बना रही थी, प्रेशर कुकर में दाल जल्दी गल जाती है।"
-बेटा अमन... [annoyed] "मैं फ़्रिज में बर्फ़ जमा रहा था। पानी शून्य डिग्री पर जमता है।"
-ट्यूशन स्टूडेंट कृतिका... [calm] "मैं होमवर्क कर रही थी। पृथ्वी सूरज का एक चक्कर लगभग तीन सौ पैंसठ दिन में लगाती है।"
-किरायेदार संजय... [calm] "मैं चाय के लिए पानी गरम कर रहा था। पचास डिग्री पर पानी उबलने लगा, तो चाय पत्ती डाल दी।"
-कामवाली शांति... [nervous] "मैं कपड़े सुखा रही थी, धूप में कपड़े जल्दी सूखते हैं।"
+घर में किताबें और ग्लोब रखे थे। शिवम ने हर चीज़ पर नज़र डाली।
+पत्नी उर्मिला... "मैं रसोई में दाल बना रही थी, प्रेशर कुकर में दाल जल्दी गल जाती है।"
+बेटा अमन... "मैं फ़्रिज में बर्फ़ जमा रहा था। पानी शून्य डिग्री पर जमता है।"
+ट्यूशन स्टूडेंट कृतिका... "मैं होमवर्क कर रही थी। पृथ्वी सूरज का एक चक्कर लगभग तीन सौ पैंसठ दिन में लगाती है।"
+किरायेदार संजय... "मैं चाय के लिए पानी गरम कर रहा था। पचास डिग्री पर पानी उबलने लगा, तो चाय पत्ती डाल दी।"
+कामवाली शांति... "मैं कपड़े सुखा रही थी, धूप में कपड़े जल्दी सूखते हैं।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2620,16 +2620,16 @@
         <is>
           <t>[whispers] नौ लोग। नौ जंगल। एक झूठी सफ़ारी।
 भोपाल। वाइल्डलाइफ़ फ़ोटोग्राफ़र इम्तियाज़ ख़ान, अपने बंगले में मरे मिले!
-[serious] मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग जंगल सफ़ारी पर थे।
+मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग जंगल सफ़ारी पर थे।
 डिटेक्टिव शिवम बंगले पहुँचे।
-[thoughtful] दीवारों पर जानवरों की तस्वीरें थीं। शिवम ने हर चीज़ पर नज़र डाली।
-असिस्टेंट रोहित... [nervous] "मैं गुजरात के गिर जंगल में था। वहाँ एशियाई शेर देखे।"
-पार्टनर विवेक... [excited] "मैं उत्तराखंड के जिम कॉर्बेट में था। जीप सफ़ारी में दो बब्बर शेर दिखे, क्या नज़ारा था!"
-पत्नी नाज़िया... [annoyed] "मैं असम के काज़ीरंगा में थी। एक सींग वाला गैंडा देखा।"
-गाइड कल्लू... [calm] "मैं राजस्थान के रणथंभौर में था, बाघ के पीछे जीप दौड़ा रहा था।"
-बेटी ज़ोया... [calm] "मैं सुंदरबन में थी। रॉयल बंगाल टाइगर के पैरों के निशान देखे।"
+दीवारों पर जानवरों की तस्वीरें थीं। शिवम ने हर चीज़ पर नज़र डाली।
+असिस्टेंट रोहित... "मैं गुजरात के गिर जंगल में था। वहाँ एशियाई शेर देखे।"
+पार्टनर विवेक... "मैं उत्तराखंड के जिम कॉर्बेट में था। जीप सफ़ारी में दो बब्बर शेर दिखे, क्या नज़ारा था!"
+पत्नी नाज़िया... "मैं असम के काज़ीरंगा में थी। एक सींग वाला गैंडा देखा।"
+गाइड कल्लू... "मैं राजस्थान के रणथंभौर में था, बाघ के पीछे जीप दौड़ा रहा था।"
+बेटी ज़ोया... "मैं सुंदरबन में थी। रॉयल बंगाल टाइगर के पैरों के निशान देखे।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2695,16 +2695,16 @@
         <is>
           <t>[whispers] नौ मुसाफ़िर। नौ सफ़र। एक नक़्शा ग़लत।
 गंगटोक। होमस्टे के मालिक छेरिंग भूटिया, अपने होमस्टे में मरे मिले!
-[serious] मौत रात आठ से नौ के बीच। सारे मेहमान बोले, हम घूमकर अभी लौटे हैं।
+मौत रात आठ से नौ के बीच। सारे मेहमान बोले, हम घूमकर अभी लौटे हैं।
 डिटेक्टिव शिवम होमस्टे पहुँचे।
-[thoughtful] होमस्टे में आग जल रही थी। शिवम ने हर चीज़ पर नज़र डाली।
-ट्रेकर अंशुल... [annoyed] "मैं लेह से लौटा हूँ। वहाँ हवा इतनी पतली है कि साँस फूल जाती है।"
-ब्लॉगर तन्वी... [calm] "मैं मेघालय के चेरापूंजी से आई, दुनिया की सबसे ज़्यादा बारिश वाली जगहों में से एक।"
-फ़ोटोग्राफ़र पार्थ... [calm] "मैं कच्छ के रण में था, सफ़ेद नमक का रेगिस्तान।"
-कुक दोरजी... [nervous] "मैं कर्नाटक के हम्पी गया था, विजयनगर साम्राज्य के खंडहर।"
-गाइड विक्रम... [calm] "मैं तो यहीं सिक्किम में नाथुला दर्रे पर टूरिस्ट ले गया था, जहाँ भारत की सीमा नेपाल से लगती है।"
+होमस्टे में आग जल रही थी। शिवम ने हर चीज़ पर नज़र डाली।
+ट्रेकर अंशुल... "मैं लेह से लौटा हूँ। वहाँ हवा इतनी पतली है कि साँस फूल जाती है।"
+ब्लॉगर तन्वी... "मैं मेघालय के चेरापूंजी से आई, दुनिया की सबसे ज़्यादा बारिश वाली जगहों में से एक।"
+फ़ोटोग्राफ़र पार्थ... "मैं कच्छ के रण में था, सफ़ेद नमक का रेगिस्तान।"
+कुक दोरजी... "मैं कर्नाटक के हम्पी गया था, विजयनगर साम्राज्य के खंडहर।"
+गाइड विक्रम... "मैं तो यहीं सिक्किम में नाथुला दर्रे पर टूरिस्ट ले गया था, जहाँ भारत की सीमा नेपाल से लगती है।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2770,16 +2770,16 @@
         <is>
           <t>[whispers] पाँच लोग। पाँच इमारतें। इतिहास झूठ नहीं बोलता।
 भुवनेश्वर। म्यूज़ियम के क्यूरेटर डॉ. बिजय महापात्रा, म्यूज़ियम हॉल में मरे मिले!
-[serious] मौत दोपहर दो से तीन के बीच। सब बोले, हम उस वक़्त अलग-अलग इमारतें देखने गए थे।
+मौत दोपहर दो से तीन के बीच। सब बोले, हम उस वक़्त अलग-अलग इमारतें देखने गए थे।
 डिटेक्टिव शिवम म्यूज़ियम पहुँचे।
-[thoughtful] हॉल में पुरानी मूर्तियाँ खड़ी थीं। शिवम ने हर चीज़ पर नज़र डाली।
-असिस्टेंट क्यूरेटर पूजा... [annoyed] "मैं कर्नाटक के बीजापुर में गोल गुम्बज देख रही थी।"
-गार्ड हरिहर... [nervous] "मैं कोलकाता के विक्टोरिया मेमोरियल गया था।"
-एंटीक डीलर मल्होत्रा... [calm] "मैं मुंबई में गेटवे ऑफ़ इंडिया पर था, जो उन्नीस सौ सैंतालीस में आज़ादी की ख़ुशी में बना था।"
-फ़ोटोग्राफ़र अनीता... [nervous] "मैं कोणार्क के सूर्य मंदिर में थी, जो रथ के आकार का है।"
-बेटा अभिजीत... [annoyed] "मैं दिल्ली में इंडिया गेट पर था, पहले विश्व युद्ध के शहीदों की याद में बना।"
+हॉल में पुरानी मूर्तियाँ खड़ी थीं। शिवम ने हर चीज़ पर नज़र डाली।
+असिस्टेंट क्यूरेटर पूजा... "मैं कर्नाटक के बीजापुर में गोल गुम्बज देख रही थी।"
+गार्ड हरिहर... "मैं कोलकाता के विक्टोरिया मेमोरियल गया था।"
+एंटीक डीलर मल्होत्रा... "मैं मुंबई में गेटवे ऑफ़ इंडिया पर था, जो उन्नीस सौ सैंतालीस में आज़ादी की ख़ुशी में बना था।"
+फ़ोटोग्राफ़र अनीता... "मैं कोणार्क के सूर्य मंदिर में थी, जो रथ के आकार का है।"
+बेटा अभिजीत... "मैं दिल्ली में इंडिया गेट पर था, पहले विश्व युद्ध के शहीदों की याद में बना।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2845,16 +2845,16 @@
         <is>
           <t>[whispers] आठ लोग। आठ रिपोर्ट। एक रिपोर्ट नक़ली।
 लुधियाना। हॉस्पिटल के मालिक डॉ. हरजीत ग्रेवाल, अपने केबिन में मरे मिले!
-[serious] मौत रात दस से ग्यारह के बीच। सब बोले, हम हॉस्पिटल के अलग-अलग विभाग में थे।
+मौत रात दस से ग्यारह के बीच। सब बोले, हम हॉस्पिटल के अलग-अलग विभाग में थे।
 डिटेक्टिव शिवम हॉस्पिटल पहुँचे।
-[thoughtful] केबिन में फ़ाइलें और दवाइयाँ बिखरी थीं। शिवम ने हर चीज़ पर नज़र डाली।
-जिम ट्रेनर जस्सी... [annoyed] "मैं हॉस्पिटल के फ़िज़ियो जिम में था। आराम में दिल एक मिनट में साठ से सौ बार धड़कता है।"
-ऑर्थो डॉक्टर बाजवा... [annoyed] "मैं एक्स-रे देख रहा था। शरीर की सबसे लंबी हड्डी जाँघ की हड्डी होती है।"
-डेंटिस्ट डॉ. रश्मि... [calm] "मैं डेंटल क्लिनिक में थी। बड़े इंसान के बत्तीस दाँत होते हैं।"
-नर्स सिमरन... [nervous] "मैं वार्ड में बुख़ार नाप रही थी। सामान्य शरीर का तापमान लगभग सैंतीस डिग्री होता है।"
-बिज़नेसमैन ढिल्लों... [calm] "मैं ब्लड बैंक में था। मेरा ग्रुप एबी पॉज़िटिव है, जो यूनिवर्सल डोनर होता है, इसलिए उन्होंने तुरंत मेरा ख़ून ले लिया।"
+केबिन में फ़ाइलें और दवाइयाँ बिखरी थीं। शिवम ने हर चीज़ पर नज़र डाली।
+जिम ट्रेनर जस्सी... "मैं हॉस्पिटल के फ़िज़ियो जिम में था। आराम में दिल एक मिनट में साठ से सौ बार धड़कता है।"
+ऑर्थो डॉक्टर बाजवा... "मैं एक्स-रे देख रहा था। शरीर की सबसे लंबी हड्डी जाँघ की हड्डी होती है।"
+डेंटिस्ट डॉ. रश्मि... "मैं डेंटल क्लिनिक में थी। बड़े इंसान के बत्तीस दाँत होते हैं।"
+नर्स सिमरन... "मैं वार्ड में बुख़ार नाप रही थी। सामान्य शरीर का तापमान लगभग सैंतीस डिग्री होता है।"
+बिज़नेसमैन ढिल्लों... "मैं ब्लड बैंक में था। मेरा ग्रुप एबी पॉज़िटिव है, जो यूनिवर्सल डोनर होता है, इसलिए उन्होंने तुरंत मेरा ख़ून ले लिया।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2920,16 +2920,16 @@
         <is>
           <t>[whispers] सबके पास पक्का बहाना... पर तारीख़ कुछ और कहती है।
 कानपुर। सेठ रामनिवास गुप्ता, अपनी गद्दी पर मरे मिले!
-[serious] मौत सुबह ग्यारह से बारह के बीच।
+मौत सुबह ग्यारह से बारह के बीच।
 डिटेक्टिव शिवम हवेली पहुँचे।
-[thoughtful] गद्दी पर बही-खाते खुले पड़े थे। शिवम ने हर चीज़ पर नज़र डाली।
-मुनीम रामदयाल... [calm] "मैं ग्यारह से बारह बजे तक एसबीआई ब्रांच में सेठ जी का कैश जमा कर रहा था। कैशियर ने पाँच मिनट में काम कर दिया।"
-बेटा अशोक... [annoyed] "मैं पंजाबी ढाबे पर मक्के की रोटी और सरसों का साग खा रहा था।"
-बहू कामिनी... [calm] "मैं उडुपी होटल में मसाला डोसा खा रही थी, कर्नाटक की ख़ास डिश।"
-भतीजा राजू... [nervous] "मैं लखनऊ गया था, टुंडे के कबाब खाने।"
-ड्राइवर शेरू... [nervous] "मैं हैदराबादी बिरयानी लेने गया था।"
+गद्दी पर बही-खाते खुले पड़े थे। शिवम ने हर चीज़ पर नज़र डाली।
+मुनीम रामदयाल... "मैं ग्यारह से बारह बजे तक एसबीआई ब्रांच में सेठ जी का कैश जमा कर रहा था। कैशियर ने पाँच मिनट में काम कर दिया।"
+बेटा अशोक... "मैं पंजाबी ढाबे पर मक्के की रोटी और सरसों का साग खा रहा था।"
+बहू कामिनी... "मैं उडुपी होटल में मसाला डोसा खा रही थी, कर्नाटक की ख़ास डिश।"
+भतीजा राजू... "मैं लखनऊ गया था, टुंडे के कबाब खाने।"
+ड्राइवर शेरू... "मैं हैदराबादी बिरयानी लेने गया था।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>
@@ -2995,16 +2995,16 @@
         <is>
           <t>[whispers] आख़िरी केस। दस लोग। आसमान सब देख रहा था।
 नैनीताल। खगोल वैज्ञानिक डॉ. प्रकाश जोशी, अपनी वेधशाला में मरे मिले!
-[serious] मौत रात नौ से दस के बीच।
+मौत रात नौ से दस के बीच।
 डिटेक्टिव शिवम वेधशाला पहुँचे।
-[thoughtful] वेधशाला में तारों के नक़्शे लगे थे। शिवम ने हर चीज़ पर नज़र डाली।
-असिस्टेंट तन्मय... [nervous] "मैं प्लैनेटेरियम में बच्चों को बता रहा था, मंगल को लाल ग्रह कहते हैं।"
-बेटी गार्गी... [calm] "मैं दूरबीन से शनि के छल्ले देख रही थी।"
-स्कूल टीचर बिष्ट... [calm] "मैं बच्चों को पढ़ा रहा था, बृहस्पति सौरमंडल का सबसे बड़ा ग्रह है।"
-इंजीनियर सुरभि... [annoyed] "मैं इसरो का वीडियो देख रही थी, चंद्रयान तीन चाँद के दक्षिणी ध्रुव के पास उतरा था।"
-पड़ोसी कुंदन... [calm] "उस रात साल की सबसे लंबी रात थी। मैं नौ से दस बजे तक छत पर बैठा तारे गिन रहा था।"
+वेधशाला में तारों के नक़्शे लगे थे। शिवम ने हर चीज़ पर नज़र डाली।
+असिस्टेंट तन्मय... "मैं प्लैनेटेरियम में बच्चों को बता रहा था, मंगल को लाल ग्रह कहते हैं।"
+बेटी गार्गी... "मैं दूरबीन से शनि के छल्ले देख रही थी।"
+स्कूल टीचर बिष्ट... "मैं बच्चों को पढ़ा रहा था, बृहस्पति सौरमंडल का सबसे बड़ा ग्रह है।"
+इंजीनियर सुरभि... "मैं इसरो का वीडियो देख रही थी, चंद्रयान तीन चाँद के दक्षिणी ध्रुव के पास उतरा था।"
+पड़ोसी कुंदन... "उस रात साल की सबसे लंबी रात थी। मैं नौ से दस बजे तक छत पर बैठा तारे गिन रहा था।"
 ⏸ 3 sec chup (Shivam soch)
-[dramatic] डिटेक्टिव शिवम ने कातिल पकड़ लिया!  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)</t>
+PAKAD_LIYA_HI (डिटेक्टिव शिवम ने कातिल पकड़ लिया!)  +  CTA_HI (आंसर कमेंट करो, सही आंसर कल पिन होगा।)  +  SIGNATURE_HI (शिवम की नज़र से कोई नहीं बचता।)  [purani files]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 4: 10 Very Hard reels (alag pattern, checklist script), reel image list fix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVfDRs8Z25TZnX8xvhD7fv
</commit_message>
<xml_diff>
--- a/youtube stories/batch 3/Batch 3 - 10 Reels.xlsx
+++ b/youtube stories/batch 3/Batch 3 - 10 Reels.xlsx
@@ -774,7 +774,7 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Reel VO poori story EK BAAR mein (Rudra, eleven_v4, stability 0.45, speed 1.05 + purana tighten). EMOTION TAG KAM SE KAM: sirf hook par [whispers], baaki saadi line – suspect ke bayaan par koi tag nahi (killer alag na lage). VO mein NAHI: 'bole/boli', motive line, galat-ishara line, saboot ka naam, 'full video/link bio'. End: 3 sec chup -&gt; PAKAD_LIYA_HI + CTA_HI + SIGNATURE_HI (purani files, dobara nahi banti).</t>
+          <t>Reel VO poori story EK BAAR mein (Rudra, eleven_v4, stability 0.45, speed 1.05 + purana tighten). EMOTION TAG KAM SE KAM: sirf hook par [whispers] + maut wali line par [serious], baaki saadi line – suspect ke bayaan par koi tag nahi (killer alag na lage). VO mein NAHI: 'bole/boli', motive line, galat-ishara line, saboot ka naam, 'full video/link bio'. End: 3 sec chup -&gt; PAKAD_LIYA_HI + CTA_HI + SIGNATURE_HI (purani files, dobara nahi banti).</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Image Prompts sheet: HARA = purani image (nayi mat banao) – 69 purani. Sirf 16 nayi banani hain: P_A021_PHOTO, P_A022_SHELL, P_A022_COCONUT, A023_GILL, P_A024_GLOBE, P_A025_LENS, P_A025_CUP, P_A027_CASE, P_A028_SYRINGE, P_A028_TEA, A028_RASHMI, A028_SIMRAN, A028_DHILLON, P_A029_CALENDAR, P_A030_CALENDAR, P_A030_LAPTOP.</t>
+          <t>Image Prompts sheet: HARA = purani image (nayi mat banao) – 79 purani. Sirf 36 nayi banani hain: P_A021_FILE, P_A021_KHIDKI, P_A021_PEN, P_A021_PHOTO, P_A022_SHELL, P_A022_KEYCARD, P_A022_SAND, P_A022_COCONUT, P_A023_LOCKER, P_A023_TOWEL, P_A023_LIST, A023_GILL, P_A024_GLOBE, P_A024_BOOK, P_A025_LENS, P_A025_CARD, P_A025_MAP, P_A025_CUP, P_A026_MAP, P_A026_SHAWL, P_A027_CASE, P_A027_STATUE, P_A027_GLOVES, P_A028_SYRINGE, P_A028_FILE, P_A028_DRAWER, P_A028_TEA, A028_RASHMI, A028_SIMRAN, A028_DHILLON, P_A029_CALENDAR, P_A029_KHATA, P_A030_CALENDAR, P_A030_LENS, P_A030_CHART, P_A030_LAPTOP.</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
         <is>
           <t>[whispers] पाँच लोग। पाँच बहाने। सिर्फ़ एक कातिल।
 रायपुर। मिल मालिक कमलेश अग्रवाल, अपने बंगले के स्टडी रूम में मरे मिले!
-मौत रात आठ से नौ के बीच। घर के सब लोग बोले, हम तो शहर से बाहर थे।
+[serious] मौत रात आठ से नौ के बीच। घर के सब लोग बोले, हम तो शहर से बाहर थे।
 डिटेक्टिव शिवम बंगले पहुँचे।
 स्टडी रूम में सफ़र की तस्वीरें लगी थीं। शिवम ने हर चीज़ पर नज़र डाली।
 बेटा राहुल... "मैं हैदराबाद में था। हुसैन सागर झील में बुद्ध की बड़ी मूर्ति के पास बोटिंग कर रहा था।"
@@ -2395,7 +2395,7 @@
         <is>
           <t>[whispers] रात नौ बजे... एक चीख़। और पाँच लोग शक के घेरे में।
 विशाखापट्टनम। रिज़ॉर्ट मालिक श्रीनिवास राव, अपने ऑफ़िस में मरे मिले!
-मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग समुंदर किनारे छुट्टी पर थे।
+[serious] मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग समुंदर किनारे छुट्टी पर थे।
 डिटेक्टिव शिवम रिज़ॉर्ट पहुँचे।
 ऑफ़िस में समुंदर की हवा आ रही थी। शिवम ने हर चीज़ पर नज़र डाली।
 पार्टनर रेड्डी... "मैं गोवा के बागा बीच पर था। अरब सागर की लहरें देख रहा था।"
@@ -2470,7 +2470,7 @@
         <is>
           <t>[whispers] पाँच चेहरे। सब मासूम दिखते हैं... एक नहीं है।
 पुणे। स्पोर्ट्स क्लब के प्रेसिडेंट विजय देशमुख, लॉकर रूम में मरे मिले!
-मौत शाम पाँच से छह के बीच। उस वक़्त क्लब में हर कोई कोई न कोई खेल खेल रहा था।
+[serious] मौत शाम पाँच से छह के बीच। उस वक़्त क्लब में हर कोई कोई न कोई खेल खेल रहा था।
 डिटेक्टिव शिवम क्लब पहुँचे।
 लॉकर रूम में ट्रॉफ़ियाँ बिखरी थीं। शिवम ने हर चीज़ पर नज़र डाली।
 हॉकी कोच गिल... "मैं मैदान पर हॉकी मैच करवा रहा था। दोनों टीमों में ग्यारह-ग्यारह खिलाड़ी।"
@@ -2545,7 +2545,7 @@
         <is>
           <t>[whispers] पाँच लोग। सबके पास पक्का बहाना। फिर कातिल कौन?
 जबलपुर। साइंस टीचर रमेश पांडे, अपने घर में मरे मिले!
-मौत रात आठ से नौ के बीच। घर के सब लोग अपने-अपने काम में लगे थे।
+[serious] मौत रात आठ से नौ के बीच। घर के सब लोग अपने-अपने काम में लगे थे।
 डिटेक्टिव शिवम घर पहुँचे।
 घर में किताबें और ग्लोब रखे थे। शिवम ने हर चीज़ पर नज़र डाली।
 पत्नी उर्मिला... "मैं रसोई में दाल बना रही थी, प्रेशर कुकर में दाल जल्दी गल जाती है।"
@@ -2620,7 +2620,7 @@
         <is>
           <t>[whispers] एक मौत। पाँच शक। और सिर्फ़ एक सच।
 भोपाल। वाइल्डलाइफ़ फ़ोटोग्राफ़र इम्तियाज़ ख़ान, अपने बंगले में मरे मिले!
-मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग जंगल सफ़ारी पर थे।
+[serious] मौत रात नौ से दस के बीच। सबने कहा, हम अलग-अलग जंगल सफ़ारी पर थे।
 डिटेक्टिव शिवम बंगले पहुँचे।
 दीवारों पर जानवरों की तस्वीरें थीं। शिवम ने हर चीज़ पर नज़र डाली।
 असिस्टेंट रोहित... "मैं गुजरात के गिर जंगल में था। वहाँ एशियाई शेर देखे।"
@@ -2695,7 +2695,7 @@
         <is>
           <t>[whispers] ध्यान से सुनना... इनमें से एक झूठ बोल रहा है।
 गंगटोक। होमस्टे के मालिक छेरिंग भूटिया, अपने होमस्टे में मरे मिले!
-मौत रात आठ से नौ के बीच। सारे मेहमान बोले, हम घूमकर अभी लौटे हैं।
+[serious] मौत रात आठ से नौ के बीच। सारे मेहमान बोले, हम घूमकर अभी लौटे हैं।
 डिटेक्टिव शिवम होमस्टे पहुँचे।
 होमस्टे में आग जल रही थी। शिवम ने हर चीज़ पर नज़र डाली।
 ट्रेकर अंशुल... "मैं लेह से लौटा हूँ। वहाँ हवा इतनी पतली है कि साँस फूल जाती है।"
@@ -2770,7 +2770,7 @@
         <is>
           <t>[whispers] पाँच लोग। पाँच कहानियाँ। एक कहानी में कातिल छुपा है।
 भुवनेश्वर। म्यूज़ियम के क्यूरेटर डॉ. बिजय महापात्रा, म्यूज़ियम हॉल में मरे मिले!
-मौत दोपहर दो से तीन के बीच। सब बोले, हम उस वक़्त अलग-अलग इमारतें देखने गए थे।
+[serious] मौत दोपहर दो से तीन के बीच। सब बोले, हम उस वक़्त अलग-अलग इमारतें देखने गए थे।
 डिटेक्टिव शिवम म्यूज़ियम पहुँचे।
 हॉल में पुरानी मूर्तियाँ खड़ी थीं। शिवम ने हर चीज़ पर नज़र डाली।
 असिस्टेंट क्यूरेटर पूजा... "मैं कर्नाटक के बीजापुर में गोल गुम्बज देख रही थी।"
@@ -2845,7 +2845,7 @@
         <is>
           <t>[whispers] निन्यानवे परसेंट लोग यहाँ ग़लत नाम लेते हैं। तुम?
 लुधियाना। हॉस्पिटल के मालिक डॉ. हरजीत ग्रेवाल, अपने केबिन में मरे मिले!
-मौत रात दस से ग्यारह के बीच। सब बोले, हम हॉस्पिटल के अलग-अलग विभाग में थे।
+[serious] मौत रात दस से ग्यारह के बीच। सब बोले, हम हॉस्पिटल के अलग-अलग विभाग में थे।
 डिटेक्टिव शिवम हॉस्पिटल पहुँचे।
 केबिन में फ़ाइलें और दवाइयाँ बिखरी थीं। शिवम ने हर चीज़ पर नज़र डाली।
 जिम ट्रेनर जस्सी... "मैं हॉस्पिटल के फ़िज़ियो जिम में था। आराम में दिल एक मिनट में साठ से सौ बार धड़कता है।"
@@ -2920,7 +2920,7 @@
         <is>
           <t>[whispers] सबसे मुश्किल केस। पाँच लोग। एक झूठ।
 कानपुर। सेठ रामनिवास गुप्ता, अपनी गद्दी पर मरे मिले!
-मौत सुबह ग्यारह से बारह के बीच।
+[serious] मौत सुबह ग्यारह से बारह के बीच।
 डिटेक्टिव शिवम हवेली पहुँचे।
 गद्दी पर बही-खाते खुले पड़े थे। शिवम ने हर चीज़ पर नज़र डाली।
 मुनीम रामदयाल... "मैं ग्यारह से बारह बजे तक एसबीआई ब्रांच में सेठ जी का कैश जमा कर रहा था। कैशियर ने पाँच मिनट में काम कर दिया।"
@@ -2995,7 +2995,7 @@
         <is>
           <t>[whispers] शिवम को बस एक लाइन लगी... तुम्हें कितनी लगेंगी?
 नैनीताल। खगोल वैज्ञानिक डॉ. प्रकाश जोशी, अपनी वेधशाला में मरे मिले!
-मौत रात नौ से दस के बीच।
+[serious] मौत रात नौ से दस के बीच।
 डिटेक्टिव शिवम वेधशाला पहुँचे।
 वेधशाला में तारों के नक़्शे लगे थे। शिवम ने हर चीज़ पर नज़र डाली।
 असिस्टेंट तन्मय... "मैं प्लैनेटेरियम में बच्चों को बता रहा था, मंगल को लाल ग्रह कहते हैं।"
@@ -22310,7 +22310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -22404,115 +22404,115 @@
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
         <is>
+          <t>P_A021_FILE</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>A021</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Open file with a torn page: 'Mill sale agreement'</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Open file with a torn page: 'Mill sale agreement'. Text on the board/paper/screen must be clearly readable exactly as written. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>P_A021_KHIDKI</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>A021</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Open window with a curtain blowing</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Open window with a curtain blowing. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>P_A021_PEN</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>A021</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Golden pen lying on the floor</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Golden pen lying on the floor. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
           <t>P_A021_PHOTO</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>A021</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Saboot (prop)</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Wall of framed travel photos of Indian monuments</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Wall of framed travel photos of Indian monuments. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>C10-008_KARAN</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>A021</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>Beta Rahul (mill bechne par jhagda)</t>
-        </is>
-      </c>
-      <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>C009_JOSHI</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>A021</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>Manager Joshi (hisaab mein gadbad)</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>G_M_YELLOW_KURTA_CUT</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>A021</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>Bhai Naresh</t>
-        </is>
-      </c>
-      <c r="E7" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>C005_VICKY_KEY_CUT</t>
+          <t>C10-008_KARAN</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
@@ -22527,7 +22527,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Driver Bablu (gaadi ki chaabi)</t>
+          <t>Beta Rahul (mill bechne par jhagda)</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
@@ -22539,7 +22539,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>C004_BEHEN</t>
+          <t>C009_JOSHI</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
@@ -22554,7 +22554,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Bhatiji Aditi</t>
+          <t>Manager Joshi (hisaab mein gadbad)</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
@@ -22566,22 +22566,22 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>C002_ARYAN</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>A022</t>
+          <t>A021</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Victim</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Indian resort owner Srinivas Rao, about 55, white shirt, slumped on an office chair, eyes closed</t>
+          <t>Bhai Naresh</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
@@ -22591,63 +22591,63 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>P_A022_SHELL</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>A022</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>Saboot (prop)</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Big sea shell used as a paperweight, cracked</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Big sea shell used as a paperweight, cracked. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>C005_VICKY_KEY_CUT</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>A021</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Driver Bablu (gaadi ki chaabi)</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>P_A022_COCONUT</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>A022</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>Saboot (prop)</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>Half drunk tender coconut with a straw</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Half drunk tender coconut with a straw. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>C004_BEHEN</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>A021</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Bhatiji Aditi</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>G_M_OLD_NOGLASSES_CUT</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
@@ -22657,12 +22657,12 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Victim</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Partner Reddy (resort ka bantwara)</t>
+          <t>Indian resort owner Srinivas Rao, about 55, white shirt, slumped on an office chair, eyes closed</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
@@ -22672,63 +22672,63 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>G_W_PINK_SUIT_CUT</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>P_A022_SHELL</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>A022</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>Beti Swati</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Big sea shell used as a paperweight, cracked</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Big sea shell used as a paperweight, cracked. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>C007_VIKRAM</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>P_A022_KEYCARD</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>A022</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Manager D'Souza</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Hotel key card on the floor</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Hotel key card on the floor. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>C010_SUNITA</t>
+          <t>P_REGISTER_TORN</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
@@ -22738,12 +22738,12 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Patni Lata (vasiyat inke naam)</t>
+          <t>Torn booking register page</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -22753,78 +22753,78 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>C015_MARCO</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>P_A022_SAND</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>A022</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Lifeguard Johnny (geele pair isi ke)</t>
-        </is>
-      </c>
-      <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Wet sandy footprints on the office floor</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Wet sandy footprints on the office floor. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>C018_SISTER</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>P_A022_COCONUT</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>A022</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Receptionist Meena</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Half drunk tender coconut with a straw</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Half drunk tender coconut with a straw. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>A023</t>
+          <t>A022</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Victim</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Indian sports club president Vijay Deshmukh, about 60, track jacket, slumped on a locker room bench, eyes closed</t>
+          <t>Partner Reddy (resort ka bantwara)</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -22836,22 +22836,22 @@
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>P_TROPHY</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>A023</t>
+          <t>A022</t>
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Saboot (prop)</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Broken trophy on the floor</t>
+          <t>Beti Swati</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
@@ -22863,22 +22863,22 @@
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>P_BOTTLE_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>A023</t>
+          <t>A022</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Saboot (prop)</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Spilled sports water bottle</t>
+          <t>Manager D'Souza</t>
         </is>
       </c>
       <c r="E21" s="19" t="inlineStr">
@@ -22888,41 +22888,41 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>A023_GILL</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>A023</t>
-        </is>
-      </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>C010_SUNITA</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>A022</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>Hockey coach Gill (chunav mein haare the)</t>
-        </is>
-      </c>
-      <c r="E22" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Sikh hockey coach about 50, track suit, whistle, hockey stick. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Patni Lata (vasiyat inke naam)</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>C18-003_PRATEEK</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>A023</t>
+          <t>A022</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
@@ -22932,7 +22932,7 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Kabaddi khiladi Bala</t>
+          <t>Lifeguard Johnny (geele pair isi ke)</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
@@ -22944,12 +22944,12 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>G_UMPIRE_CUT</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>A023</t>
+          <t>A022</t>
         </is>
       </c>
       <c r="C24" s="19" t="inlineStr">
@@ -22959,7 +22959,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Football referee Mathew</t>
+          <t>Receptionist Meena</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
@@ -22971,7 +22971,7 @@
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>C020_NOAH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
@@ -22981,12 +22981,12 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Victim</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Shatranj khiladi Vinayak (paise udhaar liye)</t>
+          <t>Indian sports club president Vijay Deshmukh, about 60, track jacket, slumped on a locker room bench, eyes closed</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
@@ -22998,7 +22998,7 @@
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>G_CIVIL_GREEN_CUT</t>
+          <t>P_TROPHY</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
@@ -23008,12 +23008,12 @@
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Volleyball captain Ajinkya</t>
+          <t>Broken trophy on the floor</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
@@ -23023,41 +23023,41 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>C04-008_GUPTA_SLUMPED</t>
-        </is>
-      </c>
-      <c r="B27" s="19" t="inlineStr">
-        <is>
-          <t>A024</t>
-        </is>
-      </c>
-      <c r="C27" s="19" t="inlineStr">
-        <is>
-          <t>Victim</t>
-        </is>
-      </c>
-      <c r="D27" s="19" t="inlineStr">
-        <is>
-          <t>Indian science teacher Ramesh Pandey, about 55, sweater, spectacles, slumped on a study chair, eyes closed</t>
-        </is>
-      </c>
-      <c r="E27" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>P_A023_LOCKER</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>A023</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>Open locker with clothes pulled out</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Open locker with clothes pulled out. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>P_A024_GLOBE</t>
+          <t>P_A023_TOWEL</t>
         </is>
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>A024</t>
+          <t>A023</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
@@ -23067,105 +23067,105 @@
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>Globe knocked off a table</t>
+          <t>Wet towel on a bench</t>
         </is>
       </c>
       <c r="E28" s="18" t="inlineStr">
         <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Globe knocked off a table. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Wet towel on a bench. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>P_BROKEN_GLASSES_CUT</t>
-        </is>
-      </c>
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>A024</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>P_A023_LIST</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>A023</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>Saboot (prop)</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
-        <is>
-          <t>Broken spectacles on the floor</t>
-        </is>
-      </c>
-      <c r="E29" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>Club election candidate list pinned on a board</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Club election candidate list pinned on a board. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>G_W_MAROON_SAREE_CUT</t>
+          <t>P_BOTTLE_CUT</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>A024</t>
+          <t>A023</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Spilled sports water bottle</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>A023_GILL</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>A023</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>Patni Urmila (beema inke naam)</t>
-        </is>
-      </c>
-      <c r="E30" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
-        </is>
-      </c>
-      <c r="B31" s="19" t="inlineStr">
-        <is>
-          <t>A024</t>
-        </is>
-      </c>
-      <c r="C31" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t>Beta Aman (bike ke paise maange)</t>
-        </is>
-      </c>
-      <c r="E31" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Hockey coach Gill (chunav mein haare the)</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Sikh hockey coach about 50, track suit, whistle, hockey stick. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>C002_RIYA_CUT</t>
+          <t>C18-003_PRATEEK</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>A024</t>
+          <t>A023</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
@@ -23175,7 +23175,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Tuition student Kritika</t>
+          <t>Kabaddi khiladi Bala</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
@@ -23187,12 +23187,12 @@
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_UMPIRE_CUT</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>A024</t>
+          <t>A023</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
@@ -23202,7 +23202,7 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Kirayedaar Sanjay</t>
+          <t>Football referee Mathew</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
@@ -23214,12 +23214,12 @@
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>G_SHANTI</t>
+          <t>C020_NOAH</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>A024</t>
+          <t>A023</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
@@ -23229,7 +23229,7 @@
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Kaamwali Shanti (lifaafa isi ne dekha tha)</t>
+          <t>Shatranj khiladi Vinayak (paise udhaar liye)</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -23241,66 +23241,66 @@
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>G_CIVIL_GREEN_CUT</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>A023</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Volleyball captain Ajinkya</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>C04-008_GUPTA_SLUMPED</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>A024</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>Indian wildlife photographer Imtiaz Khan, about 55, khaki shirt, slumped on a sofa near camera gear, eyes closed</t>
-        </is>
-      </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Indian science teacher Ramesh Pandey, about 55, sweater, spectacles, slumped on a study chair, eyes closed</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
         <is>
           <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="18" t="inlineStr">
-        <is>
-          <t>P_A025_LENS</t>
-        </is>
-      </c>
-      <c r="B36" s="18" t="inlineStr">
-        <is>
-          <t>A025</t>
-        </is>
-      </c>
-      <c r="C36" s="18" t="inlineStr">
-        <is>
-          <t>Saboot (prop)</t>
-        </is>
-      </c>
-      <c r="D36" s="18" t="inlineStr">
-        <is>
-          <t>Expensive camera lens dropped and cracked</t>
-        </is>
-      </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Expensive camera lens dropped and cracked. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>P_A025_CUP</t>
+          <t>P_A024_GLOBE</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr">
@@ -23310,34 +23310,34 @@
       </c>
       <c r="D37" s="18" t="inlineStr">
         <is>
-          <t>Cup of black coffee, cold</t>
+          <t>Globe knocked off a table</t>
         </is>
       </c>
       <c r="E37" s="18" t="inlineStr">
         <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Cup of black coffee, cold. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Globe knocked off a table. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>G_CR_ROHIT_CUT</t>
+          <t>P_DO_CHAI_UP</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>Assistant Rohit (tasveerein churane ka shak)</t>
+          <t>Two tea cups on a table, one full</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
@@ -23347,51 +23347,51 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>G_M_CAMERA_CUT</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>A025</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>Partner Vivek</t>
-        </is>
-      </c>
-      <c r="E39" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>P_A024_BOOK</t>
+        </is>
+      </c>
+      <c r="B39" s="18" t="inlineStr">
+        <is>
+          <t>A024</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>Open science book with a torn page</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Open science book with a torn page. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>P_ALMARI_KHULI</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>Patni Naziya (talaq ka case)</t>
+          <t>Pulled-out drawer, empty cash envelope</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
@@ -23403,22 +23403,22 @@
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>G_KALLU_CUT</t>
+          <t>P_BROKEN_GLASSES_CUT</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Guide Kallu</t>
+          <t>Broken spectacles on the floor</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
@@ -23430,12 +23430,12 @@
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>C011_EMMA</t>
+          <t>G_W_MAROON_SAREE_CUT</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
@@ -23445,7 +23445,7 @@
       </c>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>Beti Zoya</t>
+          <t>Patni Urmila (beema inke naam)</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
@@ -23457,12 +23457,12 @@
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>G_M_BLUE_JACKET_A_CUT</t>
+          <t>G_M_GREY_HOODIE_CUT</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>A025</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
@@ -23472,7 +23472,7 @@
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Driver Pappu (gaadi ki chaabi)</t>
+          <t>Beta Aman (bike ke paise maange)</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
@@ -23484,22 +23484,22 @@
     <row r="44">
       <c r="A44" s="19" t="inlineStr">
         <is>
-          <t>C001_VIKAS</t>
+          <t>C002_RIYA_CUT</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>A026</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Victim</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
         <is>
-          <t>Sikkimese homestay owner Tsering Bhutia, about 55, traditional bakhu dress, slumped near a fireplace, eyes closed</t>
+          <t>Tuition student Kritika</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
@@ -23511,22 +23511,22 @@
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>P_CHAI_TRAY</t>
+          <t>C001_ROHIT</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>A026</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Saboot (prop)</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Butter tea cups on a low wooden table</t>
+          <t>Kirayedaar Sanjay</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
@@ -23538,22 +23538,22 @@
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>P_SHOES</t>
+          <t>G_SHANTI</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>A026</t>
+          <t>A024</t>
         </is>
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Saboot (prop)</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>Snowy trekking shoes near the door</t>
+          <t>Kaamwali Shanti (lifaafa isi ne dekha tha)</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -23565,22 +23565,22 @@
     <row r="47">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>C006_RAJAT</t>
+          <t>G_V_MAN_CHECK_CUT</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>A026</t>
+          <t>A025</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Victim</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Trekker Anshul (paison par jhagda)</t>
+          <t>Indian wildlife photographer Imtiaz Khan, about 55, khaki shirt, slumped on a sofa near camera gear, eyes closed</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -23590,186 +23590,186 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="inlineStr">
-        <is>
-          <t>G_TANVI</t>
-        </is>
-      </c>
-      <c r="B48" s="19" t="inlineStr">
-        <is>
-          <t>A026</t>
-        </is>
-      </c>
-      <c r="C48" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D48" s="19" t="inlineStr">
-        <is>
-          <t>Blogger Tanvi</t>
-        </is>
-      </c>
-      <c r="E48" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A48" s="18" t="inlineStr">
+        <is>
+          <t>P_A025_LENS</t>
+        </is>
+      </c>
+      <c r="B48" s="18" t="inlineStr">
+        <is>
+          <t>A025</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D48" s="18" t="inlineStr">
+        <is>
+          <t>Expensive camera lens dropped and cracked</t>
+        </is>
+      </c>
+      <c r="E48" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Expensive camera lens dropped and cracked. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>G_M_BROWN_JACKET_CUT</t>
-        </is>
-      </c>
-      <c r="B49" s="19" t="inlineStr">
-        <is>
-          <t>A026</t>
-        </is>
-      </c>
-      <c r="C49" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Photographer Parth</t>
-        </is>
-      </c>
-      <c r="E49" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A49" s="18" t="inlineStr">
+        <is>
+          <t>P_A025_CARD</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>A025</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Empty memory card slot in a camera</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Empty memory card slot in a camera. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="inlineStr">
-        <is>
-          <t>G_M_APRON_CUT</t>
-        </is>
-      </c>
-      <c r="B50" s="19" t="inlineStr">
-        <is>
-          <t>A026</t>
-        </is>
-      </c>
-      <c r="C50" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Cook Dorjee (daan peti ki chaabi)</t>
-        </is>
-      </c>
-      <c r="E50" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>P_A025_MAP</t>
+        </is>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>A025</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>Torn jungle map on a table</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Torn jungle map on a table. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="19" t="inlineStr">
         <is>
-          <t>G_CIVIL_BLACK_CUT</t>
+          <t>P_MUD_MARKS</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
         <is>
-          <t>A026</t>
+          <t>A025</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Muddy safari boots near the door</t>
+        </is>
+      </c>
+      <c r="E51" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="inlineStr">
+        <is>
+          <t>P_A025_CUP</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>A025</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>Cup of black coffee, cold</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Cup of black coffee, cold. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>G_CR_ROHIT_CUT</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t>A025</t>
+        </is>
+      </c>
+      <c r="C53" s="19" t="inlineStr">
+        <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Guide Vikram</t>
-        </is>
-      </c>
-      <c r="E51" s="19" t="inlineStr">
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>Assistant Rohit (tasveerein churane ka shak)</t>
+        </is>
+      </c>
+      <c r="E53" s="19" t="inlineStr">
         <is>
           <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="19" t="inlineStr">
-        <is>
-          <t>G_V_MAN_SHERWANI_CUT</t>
-        </is>
-      </c>
-      <c r="B52" s="19" t="inlineStr">
-        <is>
-          <t>A027</t>
-        </is>
-      </c>
-      <c r="C52" s="19" t="inlineStr">
-        <is>
-          <t>Victim</t>
-        </is>
-      </c>
-      <c r="D52" s="19" t="inlineStr">
-        <is>
-          <t>Indian museum curator Dr. Bijay Mohapatra, about 60, kurta and spectacles, slumped near a glass display case, eyes closed</t>
-        </is>
-      </c>
-      <c r="E52" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="18" t="inlineStr">
-        <is>
-          <t>P_A027_CASE</t>
-        </is>
-      </c>
-      <c r="B53" s="18" t="inlineStr">
-        <is>
-          <t>A027</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>Saboot (prop)</t>
-        </is>
-      </c>
-      <c r="D53" s="18" t="inlineStr">
-        <is>
-          <t>Broken glass display case, empty velvet stand</t>
-        </is>
-      </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Broken glass display case, empty velvet stand. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="19" t="inlineStr">
         <is>
-          <t>P_CCTV_MONITOR</t>
+          <t>G_M_CAMERA_CUT</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>A025</t>
         </is>
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Saboot (prop)</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>CCTV monitor showing static</t>
+          <t>Partner Vivek</t>
         </is>
       </c>
       <c r="E54" s="19" t="inlineStr">
@@ -23781,12 +23781,12 @@
     <row r="55">
       <c r="A55" s="19" t="inlineStr">
         <is>
-          <t>C019_COWORKER</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>A025</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
@@ -23796,7 +23796,7 @@
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Assistant curator Pooja (promotion ruka tha)</t>
+          <t>Patni Naziya (talaq ka case)</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
@@ -23808,12 +23808,12 @@
     <row r="56">
       <c r="A56" s="19" t="inlineStr">
         <is>
-          <t>G_M_GUARD_CUT</t>
+          <t>G_KALLU_CUT</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>A025</t>
         </is>
       </c>
       <c r="C56" s="19" t="inlineStr">
@@ -23823,7 +23823,7 @@
       </c>
       <c r="D56" s="19" t="inlineStr">
         <is>
-          <t>Guard Harihar (chaabiyan iske paas)</t>
+          <t>Guide Kallu</t>
         </is>
       </c>
       <c r="E56" s="19" t="inlineStr">
@@ -23835,12 +23835,12 @@
     <row r="57">
       <c r="A57" s="19" t="inlineStr">
         <is>
-          <t>C017_BESTMAN</t>
+          <t>C011_EMMA</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>A025</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
@@ -23850,7 +23850,7 @@
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Antique dealer Malhotra</t>
+          <t>Beti Zoya</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
@@ -23862,12 +23862,12 @@
     <row r="58">
       <c r="A58" s="19" t="inlineStr">
         <is>
-          <t>C010_SUNITA</t>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>A025</t>
         </is>
       </c>
       <c r="C58" s="19" t="inlineStr">
@@ -23877,7 +23877,7 @@
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>Patni Sujata (vasiyat inke naam)</t>
+          <t>Driver Pappu (gaadi ki chaabi)</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
@@ -23889,22 +23889,22 @@
     <row r="59">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>C004_BEHEN</t>
+          <t>C001_VIKAS</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>A026</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Victim</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Photographer Anita (tasveerein chori ka shak)</t>
+          <t>Sikkimese homestay owner Tsering Bhutia, about 55, traditional bakhu dress, slumped near a fireplace, eyes closed</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
@@ -23916,22 +23916,22 @@
     <row r="60">
       <c r="A60" s="19" t="inlineStr">
         <is>
-          <t>C002_KUNAL</t>
+          <t>P_CHAI_TRAY</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
         <is>
-          <t>A027</t>
+          <t>A026</t>
         </is>
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D60" s="19" t="inlineStr">
         <is>
-          <t>Beta Abhijit (paison ki tangi)</t>
+          <t>Butter tea cups on a low wooden table</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -23941,41 +23941,41 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="19" t="inlineStr">
-        <is>
-          <t>C08-007_KAPOOR</t>
-        </is>
-      </c>
-      <c r="B61" s="19" t="inlineStr">
-        <is>
-          <t>A028</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Victim</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Indian hospital owner Dr. Harjeet Grewal, about 60, white coat, slumped on his cabin chair, eyes closed</t>
-        </is>
-      </c>
-      <c r="E61" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t>P_A026_MAP</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>A026</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Torn trekking map pinned on a wall</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Torn trekking map pinned on a wall. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>P_A028_SYRINGE</t>
+          <t>P_A026_SHAWL</t>
         </is>
       </c>
       <c r="B62" s="18" t="inlineStr">
         <is>
-          <t>A028</t>
+          <t>A026</t>
         </is>
       </c>
       <c r="C62" s="18" t="inlineStr">
@@ -23985,61 +23985,61 @@
       </c>
       <c r="D62" s="18" t="inlineStr">
         <is>
-          <t>Empty syringe on a cabin desk</t>
+          <t>Torn woollen shawl on the floor</t>
         </is>
       </c>
       <c r="E62" s="18" t="inlineStr">
         <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Empty syringe on a cabin desk. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Torn woollen shawl on the floor. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="18" t="inlineStr">
-        <is>
-          <t>P_A028_TEA</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>A028</t>
-        </is>
-      </c>
-      <c r="C63" s="18" t="inlineStr">
+      <c r="A63" s="19" t="inlineStr">
+        <is>
+          <t>P_DONATION_BOX_CUT</t>
+        </is>
+      </c>
+      <c r="B63" s="19" t="inlineStr">
+        <is>
+          <t>A026</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
         <is>
           <t>Saboot (prop)</t>
         </is>
       </c>
-      <c r="D63" s="18" t="inlineStr">
-        <is>
-          <t>Cup of tea with a lipstick mark</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Cup of tea with a lipstick mark. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Open donation box, empty</t>
+        </is>
+      </c>
+      <c r="E63" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="19" t="inlineStr">
         <is>
-          <t>C018_BOYFRIEND</t>
+          <t>P_SHOES</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>A028</t>
+          <t>A026</t>
         </is>
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
         <is>
-          <t>Gym trainer Jassi (paise udhaar liye the)</t>
+          <t>Snowy trekking shoes near the door</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -24051,12 +24051,12 @@
     <row r="65">
       <c r="A65" s="19" t="inlineStr">
         <is>
-          <t>C16-001_DRMEHTA</t>
+          <t>C006_RAJAT</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
         <is>
-          <t>A028</t>
+          <t>A026</t>
         </is>
       </c>
       <c r="C65" s="19" t="inlineStr">
@@ -24066,7 +24066,7 @@
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>Ortho doctor Bajwa (partnership ka jhagda)</t>
+          <t>Trekker Anshul (paison par jhagda)</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
@@ -24076,186 +24076,186 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="16" t="inlineStr">
-        <is>
-          <t>A028_RASHMI</t>
-        </is>
-      </c>
-      <c r="B66" s="16" t="inlineStr">
-        <is>
-          <t>A028</t>
-        </is>
-      </c>
-      <c r="C66" s="16" t="inlineStr">
+      <c r="A66" s="19" t="inlineStr">
+        <is>
+          <t>G_TANVI</t>
+        </is>
+      </c>
+      <c r="B66" s="19" t="inlineStr">
+        <is>
+          <t>A026</t>
+        </is>
+      </c>
+      <c r="C66" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>Dentist Dr. Rashmi</t>
-        </is>
-      </c>
-      <c r="E66" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian woman doctor about 35, mask on chin, dental mirror. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>Blogger Tanvi</t>
+        </is>
+      </c>
+      <c r="E66" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="16" t="inlineStr">
-        <is>
-          <t>A028_SIMRAN</t>
-        </is>
-      </c>
-      <c r="B67" s="16" t="inlineStr">
-        <is>
-          <t>A028</t>
-        </is>
-      </c>
-      <c r="C67" s="16" t="inlineStr">
+      <c r="A67" s="19" t="inlineStr">
+        <is>
+          <t>G_M_BROWN_JACKET_CUT</t>
+        </is>
+      </c>
+      <c r="B67" s="19" t="inlineStr">
+        <is>
+          <t>A026</t>
+        </is>
+      </c>
+      <c r="C67" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D67" s="16" t="inlineStr">
-        <is>
-          <t>Nurse Simran (lipstick ka nishaan)</t>
-        </is>
-      </c>
-      <c r="E67" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Punjabi nurse about 30, nurse uniform, thermometer, red lipstick. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="D67" s="19" t="inlineStr">
+        <is>
+          <t>Photographer Parth</t>
+        </is>
+      </c>
+      <c r="E67" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="16" t="inlineStr">
-        <is>
-          <t>A028_DHILLON</t>
-        </is>
-      </c>
-      <c r="B68" s="16" t="inlineStr">
-        <is>
-          <t>A028</t>
-        </is>
-      </c>
-      <c r="C68" s="16" t="inlineStr">
+      <c r="A68" s="19" t="inlineStr">
+        <is>
+          <t>G_M_APRON_CUT</t>
+        </is>
+      </c>
+      <c r="B68" s="19" t="inlineStr">
+        <is>
+          <t>A026</t>
+        </is>
+      </c>
+      <c r="C68" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
-        <is>
-          <t>Businessman Dhillon</t>
-        </is>
-      </c>
-      <c r="E68" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Punjabi businessman about 50, turban, blazer, bandage on arm, proud face. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="D68" s="19" t="inlineStr">
+        <is>
+          <t>Cook Dorjee (daan peti ki chaabi)</t>
+        </is>
+      </c>
+      <c r="E68" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="19" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>G_CIVIL_BLACK_CUT</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
         <is>
-          <t>A029</t>
+          <t>A026</t>
         </is>
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D69" s="19" t="inlineStr">
+        <is>
+          <t>Guide Vikram</t>
+        </is>
+      </c>
+      <c r="E69" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="19" t="inlineStr">
+        <is>
+          <t>G_V_MAN_SHERWANI_CUT</t>
+        </is>
+      </c>
+      <c r="B70" s="19" t="inlineStr">
+        <is>
+          <t>A027</t>
+        </is>
+      </c>
+      <c r="C70" s="19" t="inlineStr">
+        <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D69" s="19" t="inlineStr">
-        <is>
-          <t>Indian merchant Seth Ramniwas Gupta, about 65, dhoti kurta, slumped at a ledger desk, eyes closed</t>
-        </is>
-      </c>
-      <c r="E69" s="19" t="inlineStr">
+      <c r="D70" s="19" t="inlineStr">
+        <is>
+          <t>Indian museum curator Dr. Bijay Mohapatra, about 60, kurta and spectacles, slumped near a glass display case, eyes closed</t>
+        </is>
+      </c>
+      <c r="E70" s="19" t="inlineStr">
         <is>
           <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="18" t="inlineStr">
-        <is>
-          <t>P_A029_CALENDAR</t>
-        </is>
-      </c>
-      <c r="B70" s="18" t="inlineStr">
-        <is>
-          <t>A029</t>
-        </is>
-      </c>
-      <c r="C70" s="18" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="18" t="inlineStr">
+        <is>
+          <t>P_A027_CASE</t>
+        </is>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>A027</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
         <is>
           <t>Saboot (prop)</t>
         </is>
       </c>
-      <c r="D70" s="18" t="inlineStr">
-        <is>
-          <t>Wall calendar showing the month of October with the date 2 circled in red (no festival names written)</t>
-        </is>
-      </c>
-      <c r="E70" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Wall calendar showing the month of October with the date 2 circled in red (no festival names written). Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="19" t="inlineStr">
-        <is>
-          <t>P_BROKEN_GLASSES_CUT</t>
-        </is>
-      </c>
-      <c r="B71" s="19" t="inlineStr">
-        <is>
-          <t>A029</t>
-        </is>
-      </c>
-      <c r="C71" s="19" t="inlineStr">
-        <is>
-          <t>Saboot (prop)</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>Broken spectacles on the gaddi</t>
-        </is>
-      </c>
-      <c r="E71" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Broken glass display case, empty velvet stand</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Broken glass display case, empty velvet stand. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="19" t="inlineStr">
         <is>
-          <t>G_M_OLD_NOGLASSES_CUT</t>
+          <t>P_VISITOR_REGISTER</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
         <is>
-          <t>A029</t>
+          <t>A027</t>
         </is>
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
         <is>
-          <t>Munim Ramdayal</t>
+          <t>Visitor register with a torn page</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
@@ -24265,78 +24265,78 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="19" t="inlineStr">
-        <is>
-          <t>C003_BHATIJA</t>
-        </is>
-      </c>
-      <c r="B73" s="19" t="inlineStr">
-        <is>
-          <t>A029</t>
-        </is>
-      </c>
-      <c r="C73" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D73" s="19" t="inlineStr">
-        <is>
-          <t>Beta Ashok (gaddi ka jhagda)</t>
-        </is>
-      </c>
-      <c r="E73" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A73" s="18" t="inlineStr">
+        <is>
+          <t>P_A027_STATUE</t>
+        </is>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>A027</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Small stone statue lying on the floor</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Small stone statue lying on the floor. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="19" t="inlineStr">
-        <is>
-          <t>C002_POOJA</t>
-        </is>
-      </c>
-      <c r="B74" s="19" t="inlineStr">
-        <is>
-          <t>A029</t>
-        </is>
-      </c>
-      <c r="C74" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D74" s="19" t="inlineStr">
-        <is>
-          <t>Bahu Kamini</t>
-        </is>
-      </c>
-      <c r="E74" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A74" s="18" t="inlineStr">
+        <is>
+          <t>P_A027_GLOVES</t>
+        </is>
+      </c>
+      <c r="B74" s="18" t="inlineStr">
+        <is>
+          <t>A027</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>Pair of white cotton gloves</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Pair of white cotton gloves. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="19" t="inlineStr">
         <is>
-          <t>C004_AMIT</t>
+          <t>P_CCTV_MONITOR</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
         <is>
-          <t>A029</t>
+          <t>A027</t>
         </is>
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Saboot (prop)</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
         <is>
-          <t>Bhatija Raju (udhaar nahi lautaya)</t>
+          <t>CCTV monitor showing static</t>
         </is>
       </c>
       <c r="E75" s="19" t="inlineStr">
@@ -24348,12 +24348,12 @@
     <row r="76">
       <c r="A76" s="19" t="inlineStr">
         <is>
-          <t>G_M_BLUE_JACKET_A_CUT</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
         <is>
-          <t>A029</t>
+          <t>A027</t>
         </is>
       </c>
       <c r="C76" s="19" t="inlineStr">
@@ -24363,7 +24363,7 @@
       </c>
       <c r="D76" s="19" t="inlineStr">
         <is>
-          <t>Driver Sheru (tijori ke paas iske joote)</t>
+          <t>Assistant curator Pooja (promotion ruka tha)</t>
         </is>
       </c>
       <c r="E76" s="19" t="inlineStr">
@@ -24375,22 +24375,22 @@
     <row r="77">
       <c r="A77" s="19" t="inlineStr">
         <is>
-          <t>C04-010_ARJUN</t>
+          <t>G_M_GUARD_CUT</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
         <is>
-          <t>A030</t>
+          <t>A027</t>
         </is>
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Victim</t>
+          <t>Suspect</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
         <is>
-          <t>Indian astronomer Dr. Prakash Joshi, about 62, woollen sweater, slumped near a telescope, eyes closed</t>
+          <t>Guard Harihar (chaabiyan iske paas)</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
@@ -24400,68 +24400,68 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="18" t="inlineStr">
-        <is>
-          <t>P_A030_CALENDAR</t>
-        </is>
-      </c>
-      <c r="B78" s="18" t="inlineStr">
-        <is>
-          <t>A030</t>
-        </is>
-      </c>
-      <c r="C78" s="18" t="inlineStr">
-        <is>
-          <t>Saboot (prop)</t>
-        </is>
-      </c>
-      <c r="D78" s="18" t="inlineStr">
-        <is>
-          <t>Desk calendar showing 'JUNE' with the date 21 circled (no other words)</t>
-        </is>
-      </c>
-      <c r="E78" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Desk calendar showing 'JUNE' with the date 21 circled (no other words). Text on the board/paper/screen must be clearly readable exactly as written. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="A78" s="19" t="inlineStr">
+        <is>
+          <t>C017_BESTMAN</t>
+        </is>
+      </c>
+      <c r="B78" s="19" t="inlineStr">
+        <is>
+          <t>A027</t>
+        </is>
+      </c>
+      <c r="C78" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D78" s="19" t="inlineStr">
+        <is>
+          <t>Antique dealer Malhotra</t>
+        </is>
+      </c>
+      <c r="E78" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="18" t="inlineStr">
-        <is>
-          <t>P_A030_LAPTOP</t>
-        </is>
-      </c>
-      <c r="B79" s="18" t="inlineStr">
-        <is>
-          <t>A030</t>
-        </is>
-      </c>
-      <c r="C79" s="18" t="inlineStr">
-        <is>
-          <t>Saboot (prop)</t>
-        </is>
-      </c>
-      <c r="D79" s="18" t="inlineStr">
-        <is>
-          <t>Laptop showing a blurry photo of the moon</t>
-        </is>
-      </c>
-      <c r="E79" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Laptop showing a blurry photo of the moon. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="A79" s="19" t="inlineStr">
+        <is>
+          <t>C010_SUNITA</t>
+        </is>
+      </c>
+      <c r="B79" s="19" t="inlineStr">
+        <is>
+          <t>A027</t>
+        </is>
+      </c>
+      <c r="C79" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="inlineStr">
+        <is>
+          <t>Patni Sujata (vasiyat inke naam)</t>
+        </is>
+      </c>
+      <c r="E79" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="19" t="inlineStr">
         <is>
-          <t>C020_BROTHER</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
         <is>
-          <t>A030</t>
+          <t>A027</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
@@ -24471,7 +24471,7 @@
       </c>
       <c r="D80" s="19" t="inlineStr">
         <is>
-          <t>Assistant Tanmay (research chori ka shak)</t>
+          <t>Photographer Anita (tasveerein chori ka shak)</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
@@ -24483,12 +24483,12 @@
     <row r="81">
       <c r="A81" s="19" t="inlineStr">
         <is>
-          <t>G_W_PINK_SUIT_CUT</t>
+          <t>C002_KUNAL</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
         <is>
-          <t>A030</t>
+          <t>A027</t>
         </is>
       </c>
       <c r="C81" s="19" t="inlineStr">
@@ -24498,7 +24498,7 @@
       </c>
       <c r="D81" s="19" t="inlineStr">
         <is>
-          <t>Beti Gargi</t>
+          <t>Beta Abhijit (paison ki tangi)</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -24510,22 +24510,22 @@
     <row r="82">
       <c r="A82" s="19" t="inlineStr">
         <is>
-          <t>C011_TOM</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
         <is>
-          <t>A030</t>
+          <t>A028</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Suspect</t>
+          <t>Victim</t>
         </is>
       </c>
       <c r="D82" s="19" t="inlineStr">
         <is>
-          <t>School teacher Bisht</t>
+          <t>Indian hospital owner Dr. Harjeet Grewal, about 60, white coat, slumped on his cabin chair, eyes closed</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
@@ -24535,108 +24535,918 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="19" t="inlineStr">
-        <is>
-          <t>C018_SISTER</t>
-        </is>
-      </c>
-      <c r="B83" s="19" t="inlineStr">
-        <is>
-          <t>A030</t>
-        </is>
-      </c>
-      <c r="C83" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D83" s="19" t="inlineStr">
-        <is>
-          <t>Engineer Surabhi (project se nikaali gayi)</t>
-        </is>
-      </c>
-      <c r="E83" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A83" s="18" t="inlineStr">
+        <is>
+          <t>P_A028_SYRINGE</t>
+        </is>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
+        <is>
+          <t>Empty syringe on a cabin desk</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Empty syringe on a cabin desk. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="19" t="inlineStr">
-        <is>
-          <t>G_W_MAROON_SAREE_CUT</t>
-        </is>
-      </c>
-      <c r="B84" s="19" t="inlineStr">
-        <is>
-          <t>A030</t>
-        </is>
-      </c>
-      <c r="C84" s="19" t="inlineStr">
-        <is>
-          <t>Suspect</t>
-        </is>
-      </c>
-      <c r="D84" s="19" t="inlineStr">
-        <is>
-          <t>Patni Hemlata (beema inke naam)</t>
-        </is>
-      </c>
-      <c r="E84" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="A84" s="18" t="inlineStr">
+        <is>
+          <t>P_A028_FILE</t>
+        </is>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C84" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D84" s="18" t="inlineStr">
+        <is>
+          <t>Torn patient file</t>
+        </is>
+      </c>
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Torn patient file. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="19" t="inlineStr">
         <is>
+          <t>P_STETHOSCOPE</t>
+        </is>
+      </c>
+      <c r="B85" s="19" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C85" s="19" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
+        <is>
+          <t>Stethoscope lying on the floor</t>
+        </is>
+      </c>
+      <c r="E85" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="18" t="inlineStr">
+        <is>
+          <t>P_A028_DRAWER</t>
+        </is>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
+        <is>
+          <t>Medicine drawer pulled open</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Medicine drawer pulled open. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="18" t="inlineStr">
+        <is>
+          <t>P_A028_TEA</t>
+        </is>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>Cup of tea with a lipstick mark</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Cup of tea with a lipstick mark. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="19" t="inlineStr">
+        <is>
+          <t>C018_BOYFRIEND</t>
+        </is>
+      </c>
+      <c r="B88" s="19" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D88" s="19" t="inlineStr">
+        <is>
+          <t>Gym trainer Jassi (paise udhaar liye the)</t>
+        </is>
+      </c>
+      <c r="E88" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="19" t="inlineStr">
+        <is>
+          <t>C16-001_DRMEHTA</t>
+        </is>
+      </c>
+      <c r="B89" s="19" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C89" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D89" s="19" t="inlineStr">
+        <is>
+          <t>Ortho doctor Bajwa (partnership ka jhagda)</t>
+        </is>
+      </c>
+      <c r="E89" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="inlineStr">
+        <is>
+          <t>A028_RASHMI</t>
+        </is>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>Dentist Dr. Rashmi</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian woman doctor about 35, mask on chin, dental mirror. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>A028_SIMRAN</t>
+        </is>
+      </c>
+      <c r="B91" s="16" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="inlineStr">
+        <is>
+          <t>Nurse Simran (lipstick ka nishaan)</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Punjabi nurse about 30, nurse uniform, thermometer, red lipstick. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="inlineStr">
+        <is>
+          <t>A028_DHILLON</t>
+        </is>
+      </c>
+      <c r="B92" s="16" t="inlineStr">
+        <is>
+          <t>A028</t>
+        </is>
+      </c>
+      <c r="C92" s="16" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D92" s="16" t="inlineStr">
+        <is>
+          <t>Businessman Dhillon</t>
+        </is>
+      </c>
+      <c r="E92" s="16" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Punjabi businessman about 50, turban, blazer, bandage on arm, proud face. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="19" t="inlineStr">
+        <is>
+          <t>C17-001_SETH</t>
+        </is>
+      </c>
+      <c r="B93" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C93" s="19" t="inlineStr">
+        <is>
+          <t>Victim</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>Indian merchant Seth Ramniwas Gupta, about 65, dhoti kurta, slumped at a ledger desk, eyes closed</t>
+        </is>
+      </c>
+      <c r="E93" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="18" t="inlineStr">
+        <is>
+          <t>P_A029_CALENDAR</t>
+        </is>
+      </c>
+      <c r="B94" s="18" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>Wall calendar showing the month of October with the date 2 circled in red (no festival names written)</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Wall calendar showing the month of October with the date 2 circled in red (no festival names written). Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="19" t="inlineStr">
+        <is>
+          <t>P_TIJORI</t>
+        </is>
+      </c>
+      <c r="B95" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C95" s="19" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D95" s="19" t="inlineStr">
+        <is>
+          <t>Open iron safe with scattered cash bundles</t>
+        </is>
+      </c>
+      <c r="E95" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="18" t="inlineStr">
+        <is>
+          <t>P_A029_KHATA</t>
+        </is>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D96" s="18" t="inlineStr">
+        <is>
+          <t>Red bahi-khata ledger open with a torn page</t>
+        </is>
+      </c>
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Red bahi-khata ledger open with a torn page. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="19" t="inlineStr">
+        <is>
+          <t>P_THAALI_LASSI</t>
+        </is>
+      </c>
+      <c r="B97" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C97" s="19" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="inlineStr">
+        <is>
+          <t>Glass of lassi, half drunk</t>
+        </is>
+      </c>
+      <c r="E97" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="19" t="inlineStr">
+        <is>
+          <t>P_BROKEN_GLASSES_CUT</t>
+        </is>
+      </c>
+      <c r="B98" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C98" s="19" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D98" s="19" t="inlineStr">
+        <is>
+          <t>Broken spectacles on the gaddi</t>
+        </is>
+      </c>
+      <c r="E98" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="19" t="inlineStr">
+        <is>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
+        </is>
+      </c>
+      <c r="B99" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C99" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D99" s="19" t="inlineStr">
+        <is>
+          <t>Munim Ramdayal</t>
+        </is>
+      </c>
+      <c r="E99" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="19" t="inlineStr">
+        <is>
+          <t>C003_BHATIJA</t>
+        </is>
+      </c>
+      <c r="B100" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C100" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D100" s="19" t="inlineStr">
+        <is>
+          <t>Beta Ashok (gaddi ka jhagda)</t>
+        </is>
+      </c>
+      <c r="E100" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="19" t="inlineStr">
+        <is>
+          <t>C002_POOJA</t>
+        </is>
+      </c>
+      <c r="B101" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C101" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D101" s="19" t="inlineStr">
+        <is>
+          <t>Bahu Kamini</t>
+        </is>
+      </c>
+      <c r="E101" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="19" t="inlineStr">
+        <is>
+          <t>C004_AMIT</t>
+        </is>
+      </c>
+      <c r="B102" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C102" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D102" s="19" t="inlineStr">
+        <is>
+          <t>Bhatija Raju (udhaar nahi lautaya)</t>
+        </is>
+      </c>
+      <c r="E102" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="19" t="inlineStr">
+        <is>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
+        </is>
+      </c>
+      <c r="B103" s="19" t="inlineStr">
+        <is>
+          <t>A029</t>
+        </is>
+      </c>
+      <c r="C103" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D103" s="19" t="inlineStr">
+        <is>
+          <t>Driver Sheru (tijori ke paas iske joote)</t>
+        </is>
+      </c>
+      <c r="E103" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="19" t="inlineStr">
+        <is>
+          <t>C04-010_ARJUN</t>
+        </is>
+      </c>
+      <c r="B104" s="19" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C104" s="19" t="inlineStr">
+        <is>
+          <t>Victim</t>
+        </is>
+      </c>
+      <c r="D104" s="19" t="inlineStr">
+        <is>
+          <t>Indian astronomer Dr. Prakash Joshi, about 62, woollen sweater, slumped near a telescope, eyes closed</t>
+        </is>
+      </c>
+      <c r="E104" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="18" t="inlineStr">
+        <is>
+          <t>P_A030_CALENDAR</t>
+        </is>
+      </c>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D105" s="18" t="inlineStr">
+        <is>
+          <t>Desk calendar showing 'JUNE' with the date 21 circled (no other words)</t>
+        </is>
+      </c>
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Desk calendar showing 'JUNE' with the date 21 circled (no other words). Text on the board/paper/screen must be clearly readable exactly as written. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="18" t="inlineStr">
+        <is>
+          <t>P_A030_LENS</t>
+        </is>
+      </c>
+      <c r="B106" s="18" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D106" s="18" t="inlineStr">
+        <is>
+          <t>Telescope lens cap on the floor</t>
+        </is>
+      </c>
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Telescope lens cap on the floor. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="18" t="inlineStr">
+        <is>
+          <t>P_A030_CHART</t>
+        </is>
+      </c>
+      <c r="B107" s="18" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C107" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D107" s="18" t="inlineStr">
+        <is>
+          <t>Torn star chart</t>
+        </is>
+      </c>
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Torn star chart. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="19" t="inlineStr">
+        <is>
+          <t>P_STEEL_THERMOS</t>
+        </is>
+      </c>
+      <c r="B108" s="19" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C108" s="19" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D108" s="19" t="inlineStr">
+        <is>
+          <t>Coffee flask knocked over</t>
+        </is>
+      </c>
+      <c r="E108" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="18" t="inlineStr">
+        <is>
+          <t>P_A030_LAPTOP</t>
+        </is>
+      </c>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C109" s="18" t="inlineStr">
+        <is>
+          <t>Saboot (prop)</t>
+        </is>
+      </c>
+      <c r="D109" s="18" t="inlineStr">
+        <is>
+          <t>Laptop showing a blurry photo of the moon</t>
+        </is>
+      </c>
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Laptop showing a blurry photo of the moon. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="19" t="inlineStr">
+        <is>
+          <t>C020_BROTHER</t>
+        </is>
+      </c>
+      <c r="B110" s="19" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C110" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D110" s="19" t="inlineStr">
+        <is>
+          <t>Assistant Tanmay (research chori ka shak)</t>
+        </is>
+      </c>
+      <c r="E110" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="19" t="inlineStr">
+        <is>
+          <t>G_W_PINK_SUIT_CUT</t>
+        </is>
+      </c>
+      <c r="B111" s="19" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C111" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D111" s="19" t="inlineStr">
+        <is>
+          <t>Beti Gargi</t>
+        </is>
+      </c>
+      <c r="E111" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="19" t="inlineStr">
+        <is>
+          <t>C011_TOM</t>
+        </is>
+      </c>
+      <c r="B112" s="19" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C112" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D112" s="19" t="inlineStr">
+        <is>
+          <t>School teacher Bisht</t>
+        </is>
+      </c>
+      <c r="E112" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="19" t="inlineStr">
+        <is>
+          <t>C018_SISTER</t>
+        </is>
+      </c>
+      <c r="B113" s="19" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C113" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D113" s="19" t="inlineStr">
+        <is>
+          <t>Engineer Surabhi (project se nikaali gayi)</t>
+        </is>
+      </c>
+      <c r="E113" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="19" t="inlineStr">
+        <is>
+          <t>G_W_MAROON_SAREE_CUT</t>
+        </is>
+      </c>
+      <c r="B114" s="19" t="inlineStr">
+        <is>
+          <t>A030</t>
+        </is>
+      </c>
+      <c r="C114" s="19" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="D114" s="19" t="inlineStr">
+        <is>
+          <t>Patni Hemlata (beema inke naam)</t>
+        </is>
+      </c>
+      <c r="E114" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="19" t="inlineStr">
+        <is>
           <t>G_M_CAMERA_CUT</t>
         </is>
       </c>
-      <c r="B85" s="19" t="inlineStr">
+      <c r="B115" s="19" t="inlineStr">
         <is>
           <t>A030</t>
         </is>
       </c>
-      <c r="C85" s="19" t="inlineStr">
+      <c r="C115" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D85" s="19" t="inlineStr">
+      <c r="D115" s="19" t="inlineStr">
         <is>
           <t>Photographer Hrithik</t>
         </is>
       </c>
-      <c r="E85" s="19" t="inlineStr">
+      <c r="E115" s="19" t="inlineStr">
         <is>
           <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="19" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="19" t="inlineStr">
         <is>
           <t>C008_GUEST</t>
         </is>
       </c>
-      <c r="B86" s="19" t="inlineStr">
+      <c r="B116" s="19" t="inlineStr">
         <is>
           <t>A030</t>
         </is>
       </c>
-      <c r="C86" s="19" t="inlineStr">
+      <c r="C116" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D86" s="19" t="inlineStr">
+      <c r="D116" s="19" t="inlineStr">
         <is>
           <t>Padosi Kundan</t>
         </is>
       </c>
-      <c r="E86" s="19" t="inlineStr">
+      <c r="E116" s="19" t="inlineStr">
         <is>
           <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>

</xml_diff>